<commit_message>
Translate the field report into Tamil
The first author, a native Tamil speaker, translated all 41 sentences;
import_translation.py checks every row (numbers, placeholders, bracketed
markers) and writes configs/report_translations_ta.yaml. Each entry keeps the
English it was made from and is used only while that English is unchanged;
otherwise the sentence falls back to English under a 'not fully translated'
notice. The English report is byte-identical except for one added line, the
translator's plain explanation of the AUROC sentence (D9b), now in both
languages. Seven new tests: safety sentences in Tamil, numbers unchanged,
wording invariant to the estimate, stale-translation fallback, no stale
entries, and English blocks matching the translated sentences.
</commit_message>
<xml_diff>
--- a/translation/SICKLE-Guard_report_Tamil_translation.xlsx
+++ b/translation/SICKLE-Guard_report_Tamil_translation.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report (Tamil)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Translate'!$A$1:$I$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Translate'!$A$1:$I$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -588,7 +588,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Every sentence a farmer can see in the SICKLE-Guard field report, in the order it appears. 12 headings and labels already have a Tamil version; every sentence below them, including every safety warning, is still in English. The report will not be offered in Tamil until a native speaker has translated and checked it.</t>
+          <t>Every sentence a farmer can see in the SICKLE-Guard field report, in the order it appears. 42 of 42 already have a valid Tamil version (column F); use this sheet to review or revise them, or to translate any that are missing. The report will not be offered in Tamil until a native speaker has translated and checked it.</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -969,7 +969,11 @@
           <t>kg/acre</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr"/>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>கிலோ / ஏக்கர்</t>
+        </is>
+      </c>
       <c r="G7" s="11" t="inlineStr"/>
       <c r="H7" s="11" t="inlineStr"/>
       <c r="I7" s="9" t="inlineStr">
@@ -1002,7 +1006,7 @@
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>அடிப்படை</t>
+          <t>இதன் அடிப்படை</t>
         </is>
       </c>
       <c r="G8" s="11" t="inlineStr"/>
@@ -1068,7 +1072,7 @@
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>செயற்கைக்கோள் படம் (முந்தைய அறுவடை பதிவு இல்லை)</t>
+          <t>செயற்கைக்கோள் படங்கள் (முந்தைய அறுவடைப் பதிவு இல்லை)</t>
         </is>
       </c>
       <c r="G10" s="11" t="inlineStr"/>
@@ -1134,7 +1138,7 @@
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>கவனத்திற்கு குறிக்கப்பட்டுள்ளது</t>
+          <t>கவனத்திற்காகக் குறிக்கப்பட்டது</t>
         </is>
       </c>
       <c r="G12" s="11" t="inlineStr"/>
@@ -1171,7 +1175,11 @@
           <t>This field is among the lower estimates in its area. That is a reason to look, not a finding of loss.</t>
         </is>
       </c>
-      <c r="F13" s="10" t="inlineStr"/>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>இந்தப் பகுதியிலுள்ள ஒப்பீட்டளவில் குறைந்த விளைச்சல் மதிப்பீடுகளில் இந்த வயலும் ஒன்று. இதைச் சரிபார்க்க வேண்டிய காரணமாக எடுத்துக்கொள்ளுங்கள்; இழப்பு ஏற்பட்டுவிட்டது என்பதற்கான முடிவாக அல்ல.</t>
+        </is>
+      </c>
       <c r="G13" s="11" t="inlineStr"/>
       <c r="H13" s="11" t="inlineStr"/>
       <c r="I13" s="9" t="inlineStr">
@@ -1202,7 +1210,11 @@
           <t>Most fields flagged this way yield below average MOST YEARS. Being flagged is usually a statement about the land, not about this season.</t>
         </is>
       </c>
-      <c r="F14" s="10" t="inlineStr"/>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>இவ்வாறு குறிக்கப்படும் பெரும்பாலான வயல்களில், பெரும்பாலான ஆண்டுகளில் விளைச்சல் சராசரிக்குக் கீழே இருக்கும். இந்தக் குறிப்பு பொதுவாக நிலத்தின் வழக்கமான தன்மையைப் பற்றியது; இந்தப் பருவத்தில் என்ன நடந்தது என்பதைப் பற்றியது அல்ல.</t>
+        </is>
+      </c>
       <c r="G14" s="11" t="inlineStr"/>
       <c r="H14" s="11" t="inlineStr"/>
       <c r="I14" s="9" t="inlineStr">
@@ -1235,7 +1247,7 @@
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>இந்த அமைப்பால் குறிக்கப்படவில்லை</t>
+          <t>இந்த அமைப்பு இந்த வயலைக் குறிக்கவில்லை.</t>
         </is>
       </c>
       <c r="G15" s="11" t="inlineStr"/>
@@ -1268,7 +1280,11 @@
           <t>THIS IS NOT EVIDENCE THAT YOUR CROP IS FINE.</t>
         </is>
       </c>
-      <c r="F16" s="10" t="inlineStr"/>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>உங்கள் பயிர் நன்றாக உள்ளது என்பதற்கான ஆதாரம் இது அல்ல.</t>
+        </is>
+      </c>
       <c r="G16" s="11" t="inlineStr"/>
       <c r="H16" s="11" t="inlineStr"/>
       <c r="I16" s="9" t="inlineStr">
@@ -1303,7 +1319,11 @@
           <t>This system misses losses. If you think your crop was damaged, report it anyway.</t>
         </is>
       </c>
-      <c r="F17" s="10" t="inlineStr"/>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>இந்த அமைப்பு பயிர் இழப்புகளைத் தவறவிடுகிறது. உங்கள் பயிர் சேதமடைந்ததாக நீங்கள் நினைத்தால், இருந்தாலும் அதைத் தெரிவியுங்கள்.</t>
+        </is>
+      </c>
       <c r="G17" s="11" t="inlineStr"/>
       <c r="H17" s="11" t="inlineStr"/>
       <c r="I17" s="9" t="inlineStr"/>
@@ -1365,7 +1385,11 @@
           <t>Moderate. Built from this field's own past harvests, which on test data predicted yield far better than the satellite model (error 200 vs 346 kg/acre).</t>
         </is>
       </c>
-      <c r="F19" s="10" t="inlineStr"/>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>மிதமான நம்பகத்தன்மை. இந்த வயலின் முந்தைய அறுவடைகளை அடிப்படையாகக் கொண்டது. சோதனைத் தரவுகளில், இது செயற்கைக்கோள் மாதிரியை விட விளைச்சலை மிகவும் நன்றாகக் கணித்தது (பிழை 200 எதிராக 346 கிலோ/ஏக்கர்).</t>
+        </is>
+      </c>
       <c r="G19" s="11" t="inlineStr"/>
       <c r="H19" s="11" t="inlineStr"/>
       <c r="I19" s="9" t="inlineStr">
@@ -1400,7 +1424,11 @@
           <t>NO RELIABLE ESTIMATE.</t>
         </is>
       </c>
-      <c r="F20" s="10" t="inlineStr"/>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>நம்பகமான மதிப்பீடு இல்லை.</t>
+        </is>
+      </c>
       <c r="G20" s="11" t="inlineStr"/>
       <c r="H20" s="11" t="inlineStr"/>
       <c r="I20" s="9" t="inlineStr">
@@ -1431,7 +1459,11 @@
           <t>No past harvest on record, so the figure above is a satellite guess.</t>
         </is>
       </c>
-      <c r="F21" s="10" t="inlineStr"/>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>முந்தைய அறுவடைப் பதிவு இல்லை; எனவே மேலே உள்ள எண் செயற்கைக்கோள் தரவின் அடிப்படையிலான ஒரு கணிப்பு மட்டுமே.</t>
+        </is>
+      </c>
       <c r="G21" s="11" t="inlineStr"/>
       <c r="H21" s="11" t="inlineStr"/>
       <c r="I21" s="9" t="inlineStr"/>
@@ -1458,7 +1490,11 @@
           <t>On test data it was NOT shown to beat simply using the area average (gain 14 kg/acre, interval -30 to +4, includes zero).</t>
         </is>
       </c>
-      <c r="F22" s="10" t="inlineStr"/>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>சோதனைத் தரவுகளில், இந்தக் கணிப்பு பகுதியின் சராசரி விளைச்சலை மட்டும் பயன்படுத்துவதை விடச் சிறந்தது என்று நிரூபிக்கப்படவில்லை (முன்னேற்றம் 14 கிலோ/ஏக்கர்; இடைவெளி -30 முதல் +4 வரை; இதில் பூஜ்ஜியம் அடங்குகிறது).</t>
+        </is>
+      </c>
       <c r="G22" s="11" t="inlineStr"/>
       <c r="H22" s="11" t="inlineStr"/>
       <c r="I22" s="9" t="inlineStr">
@@ -1493,7 +1529,11 @@
           <t>Do not act on the number itself.</t>
         </is>
       </c>
-      <c r="F23" s="10" t="inlineStr"/>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>இந்த எண்ணை மட்டும் வைத்து எந்த முடிவும் எடுக்க வேண்டாம்.</t>
+        </is>
+      </c>
       <c r="G23" s="11" t="inlineStr"/>
       <c r="H23" s="11" t="inlineStr"/>
       <c r="I23" s="9" t="inlineStr"/>
@@ -1520,7 +1560,11 @@
           <t>This warning means there is NO RECORD for this field. It does NOT mean this estimate is worse than the ones without the warning: tested, the difference in error is +41 kg/acre, interval -58 to +130, which includes zero.</t>
         </is>
       </c>
-      <c r="F24" s="10" t="inlineStr"/>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>இந்த எச்சரிக்கை இந்த வயலுக்கு முந்தைய அறுவடைப் பதிவு இல்லை என்பதைக் குறிக்கிறது. எச்சரிக்கை இல்லாத வயல்களைவிட இந்த மதிப்பீடு மோசமானது என்று இதன் பொருள் அல்ல: சோதனையில் பிழை வித்தியாசம் +41 கிலோ/ஏக்கர்; இடைவெளி -58 முதல் +130 வரை, இதில் பூஜ்ஜியம் அடங்குகிறது.</t>
+        </is>
+      </c>
       <c r="G24" s="11" t="inlineStr"/>
       <c r="H24" s="11" t="inlineStr"/>
       <c r="I24" s="9" t="inlineStr">
@@ -1555,7 +1599,11 @@
           <t>This system CANNOT tell whether this particular season was bad for this field.</t>
         </is>
       </c>
-      <c r="F25" s="10" t="inlineStr"/>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>இந்த குறிப்பிட்ட வயலில் இந்தப் பருவம் மோசமாக இருந்ததா என்பதை இந்த அமைப்பால் கண்டறிய முடியாது.</t>
+        </is>
+      </c>
       <c r="G25" s="11" t="inlineStr"/>
       <c r="H25" s="11" t="inlineStr"/>
       <c r="I25" s="9" t="inlineStr"/>
@@ -1582,7 +1630,11 @@
           <t>That was tested and did not work: on fields that are sometimes below and sometimes above the threshold, ranking AUROC is 0.626 [0.386, 0.887], which includes chance.</t>
         </is>
       </c>
-      <c r="F26" s="10" t="inlineStr"/>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>இதைச் சோதித்தபோது பயனுள்ள முடிவு கிடைக்கவில்லை: சில பருவங்களில் வரம்புக்குக் கீழும் சில பருவங்களில் மேலுமாக இருக்கும் வயல்களை வரிசைப்படுத்திய மதிப்பெண் AUROC 0.626 [0.386, 0.887]. இந்த இடைவெளியில் சீரற்ற தேர்வின் அளவும் அடங்குகிறது.</t>
+        </is>
+      </c>
       <c r="G26" s="11" t="inlineStr"/>
       <c r="H26" s="11" t="inlineStr"/>
       <c r="I26" s="9" t="inlineStr">
@@ -1594,7 +1646,7 @@
     <row r="27" ht="48" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>D9b</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
@@ -1604,63 +1656,67 @@
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>report lists a rank</t>
+          <t>always</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr"/>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>Rank in this list: {rank} of {total} (lowest first).</t>
-        </is>
-      </c>
-      <c r="F27" s="10" t="inlineStr"/>
+          <t>In plain terms: this score does not reliably pick out which fields need more attention.</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>பொதுவான விளக்கம்: இந்த மதிப்பெண், எந்த வயல்களுக்கு அதிக கவனம் தேவை என்பதை நம்பகமாகத் தேர்ந்தெடுக்கவில்லை.</t>
+        </is>
+      </c>
       <c r="G27" s="11" t="inlineStr"/>
       <c r="H27" s="11" t="inlineStr"/>
       <c r="I27" s="9" t="inlineStr">
         <is>
-          <t>Keep {rank} and {total} exactly as written; the program fills them in.</t>
+          <t>Plain explanation of D9, added at the translator's suggestion.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="48" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>What to do</t>
+          <t>Trust</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>always</t>
+          <t>report lists a rank</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr"/>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>WHAT TO DO NOW</t>
+          <t>Rank in this list: {rank} of {total} (lowest first).</t>
         </is>
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
-          <t>இப்போது என்ன செய்வது</t>
+          <t>இந்தப் பட்டியலில் உள்ள இடம்: {rank} / {total} (குறைந்த மதிப்பீடு முதலில்).</t>
         </is>
       </c>
       <c r="G28" s="11" t="inlineStr"/>
       <c r="H28" s="11" t="inlineStr"/>
       <c r="I28" s="9" t="inlineStr">
         <is>
-          <t>Section heading.</t>
+          <t>Keep {rank} and {total} exactly as written; the program fills them in.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="48" customHeight="1">
-      <c r="A29" s="12" t="inlineStr">
-        <is>
-          <t>E2</t>
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>E1</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
@@ -1673,29 +1729,29 @@
           <t>always</t>
         </is>
       </c>
-      <c r="D29" s="13" t="inlineStr">
-        <is>
-          <t>SAFETY-CRITICAL</t>
-        </is>
-      </c>
-      <c r="E29" s="12" t="inlineStr">
-        <is>
-          <t>1. If your crop was damaged, report it NOW. Do not wait for any report, including this one.</t>
-        </is>
-      </c>
-      <c r="F29" s="10" t="inlineStr"/>
+      <c r="D29" s="9" t="inlineStr"/>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>WHAT TO DO NOW</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>இப்போது என்ன செய்ய வேண்டும்</t>
+        </is>
+      </c>
       <c r="G29" s="11" t="inlineStr"/>
       <c r="H29" s="11" t="inlineStr"/>
       <c r="I29" s="9" t="inlineStr">
         <is>
-          <t>The first instruction. It must stay urgent.</t>
+          <t>Section heading.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="48" customHeight="1">
-      <c r="A30" s="9" t="inlineStr">
-        <is>
-          <t>E3</t>
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>E2</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
@@ -1708,25 +1764,33 @@
           <t>always</t>
         </is>
       </c>
-      <c r="D30" s="9" t="inlineStr"/>
-      <c r="E30" s="9" t="inlineStr">
-        <is>
-          <t>localised calamity (hailstorm, landslide, inundation, cloudburst) and post-harvest loss</t>
-        </is>
-      </c>
-      <c r="F30" s="10" t="inlineStr"/>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>SAFETY-CRITICAL</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>1. If your crop was damaged, report it NOW. Do not wait for any report, including this one.</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="inlineStr">
+        <is>
+          <t>1. உங்கள் பயிர் சேதமடைந்திருந்தால், அதை இப்போதே தெரிவியுங்கள். இந்த அறிக்கை உட்பட எந்த அறிக்கைக்காகவும் காத்திருக்க வேண்டாம்.</t>
+        </is>
+      </c>
       <c r="G30" s="11" t="inlineStr"/>
       <c r="H30" s="11" t="inlineStr"/>
       <c r="I30" s="9" t="inlineStr">
         <is>
-          <t>Kind of loss this deadline applies to.</t>
+          <t>The first instruction. It must stay urgent.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="48" customHeight="1">
-      <c r="A31" s="12" t="inlineStr">
-        <is>
-          <t>E4</t>
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>E3</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
@@ -1739,29 +1803,29 @@
           <t>always</t>
         </is>
       </c>
-      <c r="D31" s="13" t="inlineStr">
-        <is>
-          <t>SAFETY-CRITICAL</t>
-        </is>
-      </c>
-      <c r="E31" s="12" t="inlineStr">
-        <is>
-          <t>report within 72 hours of the event</t>
-        </is>
-      </c>
-      <c r="F31" s="10" t="inlineStr"/>
+      <c r="D31" s="9" t="inlineStr"/>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>localised calamity (hailstorm, landslide, inundation, cloudburst) and post-harvest loss</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>உள்ளூர்மயமான பேரிடர் (ஆலங்கட்டி மழை, நிலச்சரிவு, வெள்ளநீர் புகுதல், திடீர் கனமழை) மற்றும் அறுவடைக்குப் பிந்தைய இழப்பு</t>
+        </is>
+      </c>
       <c r="G31" s="11" t="inlineStr"/>
       <c r="H31" s="11" t="inlineStr"/>
       <c r="I31" s="9" t="inlineStr">
         <is>
-          <t>Keep '72'. This deadline is not yet confirmed on an official page (see E7).</t>
+          <t>Kind of loss this deadline applies to.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="48" customHeight="1">
-      <c r="A32" s="9" t="inlineStr">
-        <is>
-          <t>E5</t>
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>E4</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
@@ -1774,21 +1838,33 @@
           <t>always</t>
         </is>
       </c>
-      <c r="D32" s="9" t="inlineStr"/>
-      <c r="E32" s="9" t="inlineStr">
-        <is>
-          <t>widespread loss across a notified area (e.g. drought, flood)</t>
-        </is>
-      </c>
-      <c r="F32" s="10" t="inlineStr"/>
+      <c r="D32" s="13" t="inlineStr">
+        <is>
+          <t>SAFETY-CRITICAL</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t>report within 72 hours of the event</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>நிகழ்வு நடந்த 72 மணி நேரத்திற்குள் தெரிவிக்கவும்</t>
+        </is>
+      </c>
       <c r="G32" s="11" t="inlineStr"/>
       <c r="H32" s="11" t="inlineStr"/>
-      <c r="I32" s="9" t="inlineStr"/>
+      <c r="I32" s="9" t="inlineStr">
+        <is>
+          <t>Keep '72'. This deadline is not yet confirmed on an official page (see E7).</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="48" customHeight="1">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>E5</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
@@ -1804,22 +1880,22 @@
       <c r="D33" s="9" t="inlineStr"/>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>no individual intimation required</t>
-        </is>
-      </c>
-      <c r="F33" s="10" t="inlineStr"/>
+          <t>widespread loss across a notified area (e.g. drought, flood)</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>அறிவிக்கப்பட்ட பகுதி முழுவதும் பரவலான இழப்பு (எ.கா., வறட்சி, வெள்ளம்)</t>
+        </is>
+      </c>
       <c r="G33" s="11" t="inlineStr"/>
       <c r="H33" s="11" t="inlineStr"/>
-      <c r="I33" s="9" t="inlineStr">
-        <is>
-          <t>'Intimation' means telling the insurer about the loss.</t>
-        </is>
-      </c>
+      <c r="I33" s="9" t="inlineStr"/>
     </row>
     <row r="34" ht="48" customHeight="1">
-      <c r="A34" s="12" t="inlineStr">
-        <is>
-          <t>E7</t>
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>E6</t>
         </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
@@ -1829,32 +1905,32 @@
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>after an unconfirmed item</t>
-        </is>
-      </c>
-      <c r="D34" s="13" t="inlineStr">
-        <is>
-          <t>SAFETY-CRITICAL</t>
-        </is>
-      </c>
-      <c r="E34" s="12" t="inlineStr">
-        <is>
-          <t>[UNVERIFIED]</t>
-        </is>
-      </c>
-      <c r="F34" s="10" t="inlineStr"/>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr"/>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>no individual intimation required</t>
+        </is>
+      </c>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>தனிப்பட்ட முறையில் தகவல் தெரிவிக்க வேண்டிய அவசியமில்லை</t>
+        </is>
+      </c>
       <c r="G34" s="11" t="inlineStr"/>
       <c r="H34" s="11" t="inlineStr"/>
       <c r="I34" s="9" t="inlineStr">
         <is>
-          <t>Marker shown after a deadline that could not be confirmed on an official page. Keep the square brackets.</t>
+          <t>'Intimation' means telling the insurer about the loss.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="48" customHeight="1">
-      <c r="A35" s="9" t="inlineStr">
-        <is>
-          <t>E8</t>
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>E7</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
@@ -1864,24 +1940,36 @@
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>always</t>
-        </is>
-      </c>
-      <c r="D35" s="9" t="inlineStr"/>
-      <c r="E35" s="9" t="inlineStr">
-        <is>
-          <t>2. Contact one of these to report or to check status:</t>
-        </is>
-      </c>
-      <c r="F35" s="10" t="inlineStr"/>
+          <t>after an unconfirmed item</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>SAFETY-CRITICAL</t>
+        </is>
+      </c>
+      <c r="E35" s="12" t="inlineStr">
+        <is>
+          <t>[UNVERIFIED]</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
+          <t>[UNVERIFIED]</t>
+        </is>
+      </c>
       <c r="G35" s="11" t="inlineStr"/>
       <c r="H35" s="11" t="inlineStr"/>
-      <c r="I35" s="9" t="inlineStr"/>
+      <c r="I35" s="9" t="inlineStr">
+        <is>
+          <t>Marker shown after a deadline that could not be confirmed on an official page. Keep the square brackets.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="48" customHeight="1">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>E9</t>
+          <t>E8</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
@@ -1897,22 +1985,22 @@
       <c r="D36" s="9" t="inlineStr"/>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>Krishi Rakshak Portal &amp; Helpline (KRPH): 14447</t>
-        </is>
-      </c>
-      <c r="F36" s="10" t="inlineStr"/>
+          <t>2. Contact one of these to report or to check status:</t>
+        </is>
+      </c>
+      <c r="F36" s="10" t="inlineStr">
+        <is>
+          <t>2. இழப்பைத் தெரிவிக்க அல்லது நிலையை அறிய, கீழே உள்ள வழிகளில் ஒன்றைத் தொடர்புகொள்ளுங்கள்:</t>
+        </is>
+      </c>
       <c r="G36" s="11" t="inlineStr"/>
       <c r="H36" s="11" t="inlineStr"/>
-      <c r="I36" s="9" t="inlineStr">
-        <is>
-          <t>Official name of the national helpline; 14447 is verified. Keep the number. Give the name as farmers would know it.</t>
-        </is>
-      </c>
+      <c r="I36" s="9" t="inlineStr"/>
     </row>
     <row r="37" ht="48" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>E10</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
@@ -1928,22 +2016,26 @@
       <c r="D37" s="9" t="inlineStr"/>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>PMFBY WhatsApp: 7065514447</t>
-        </is>
-      </c>
-      <c r="F37" s="10" t="inlineStr"/>
+          <t>Krishi Rakshak Portal &amp; Helpline (KRPH): 14447</t>
+        </is>
+      </c>
+      <c r="F37" s="10" t="inlineStr">
+        <is>
+          <t>கிருஷி ரக்ஷக் போர்டல் &amp; உதவி எண் (KRPH): 14447</t>
+        </is>
+      </c>
       <c r="G37" s="11" t="inlineStr"/>
       <c r="H37" s="11" t="inlineStr"/>
       <c r="I37" s="9" t="inlineStr">
         <is>
-          <t>Keep the number exactly.</t>
+          <t>Official name of the national helpline; 14447 is verified. Keep the number. Give the name as farmers would know it.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="48" customHeight="1">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>E11</t>
+          <t>E10</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
@@ -1959,22 +2051,26 @@
       <c r="D38" s="9" t="inlineStr"/>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>Crop Insurance mobile app: search 'Crop Insurance' by Govt. of India on the app store</t>
-        </is>
-      </c>
-      <c r="F38" s="10" t="inlineStr"/>
+          <t>PMFBY WhatsApp: 7065514447</t>
+        </is>
+      </c>
+      <c r="F38" s="10" t="inlineStr">
+        <is>
+          <t>PMFBY WhatsApp: 7065514447</t>
+        </is>
+      </c>
       <c r="G38" s="11" t="inlineStr"/>
       <c r="H38" s="11" t="inlineStr"/>
       <c r="I38" s="9" t="inlineStr">
         <is>
-          <t>'Crop Insurance' is the app's name as it appears in the app store; keep it in English so it can be searched.</t>
+          <t>Keep the number exactly.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="48" customHeight="1">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>E12</t>
+          <t>E11</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
@@ -1990,22 +2086,26 @@
       <c r="D39" s="9" t="inlineStr"/>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>Claim status: pmfby.gov.in -&gt; Farmer Corner -&gt; Application Status</t>
-        </is>
-      </c>
-      <c r="F39" s="10" t="inlineStr"/>
+          <t>Crop Insurance mobile app: search 'Crop Insurance' by Govt. of India on the app store</t>
+        </is>
+      </c>
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>மொபைல் செயலி: செயலி அங்காடியில் இந்திய அரசின் 'Crop Insurance' என்று தேடுங்கள்.</t>
+        </is>
+      </c>
       <c r="G39" s="11" t="inlineStr"/>
       <c r="H39" s="11" t="inlineStr"/>
       <c r="I39" s="9" t="inlineStr">
         <is>
-          <t>The website's menu names are in English on the site; keep 'Farmer Corner' and 'Application Status' in English, explain if needed.</t>
+          <t>'Crop Insurance' is the app's name as it appears in the app store; keep it in English so it can be searched.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="48" customHeight="1">
-      <c r="A40" s="12" t="inlineStr">
-        <is>
-          <t>E13</t>
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>E12</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
@@ -2015,32 +2115,32 @@
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>after an unconfirmed item</t>
-        </is>
-      </c>
-      <c r="D40" s="13" t="inlineStr">
-        <is>
-          <t>SAFETY-CRITICAL</t>
-        </is>
-      </c>
-      <c r="E40" s="12" t="inlineStr">
-        <is>
-          <t>[UNVERIFIED - confirm first]</t>
-        </is>
-      </c>
-      <c r="F40" s="10" t="inlineStr"/>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr"/>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>Claim status: pmfby.gov.in -&gt; Farmer Corner -&gt; Application Status</t>
+        </is>
+      </c>
+      <c r="F40" s="10" t="inlineStr">
+        <is>
+          <t>கோரிக்கை நிலை: pmfby.gov.in -&gt; Farmer Corner -&gt; Application Status</t>
+        </is>
+      </c>
       <c r="G40" s="11" t="inlineStr"/>
       <c r="H40" s="11" t="inlineStr"/>
       <c r="I40" s="9" t="inlineStr">
         <is>
-          <t>Marker after a contact that could not be confirmed. Keep the brackets.</t>
+          <t>The website's menu names are in English on the site; keep 'Farmer Corner' and 'Application Status' in English, explain if needed.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="48" customHeight="1">
-      <c r="A41" s="9" t="inlineStr">
-        <is>
-          <t>E14</t>
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>E13</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
@@ -2050,33 +2150,41 @@
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>always</t>
-        </is>
-      </c>
-      <c r="D41" s="9" t="inlineStr"/>
-      <c r="E41" s="9" t="inlineStr">
-        <is>
-          <t>3. Confirm the numbers above with your bank, the Common Service Centre, or the District Agriculture Officer. They could not be verified against an official page.</t>
-        </is>
-      </c>
-      <c r="F41" s="10" t="inlineStr"/>
+          <t>after an unconfirmed item</t>
+        </is>
+      </c>
+      <c r="D41" s="13" t="inlineStr">
+        <is>
+          <t>SAFETY-CRITICAL</t>
+        </is>
+      </c>
+      <c r="E41" s="12" t="inlineStr">
+        <is>
+          <t>[UNVERIFIED - confirm first]</t>
+        </is>
+      </c>
+      <c r="F41" s="10" t="inlineStr">
+        <is>
+          <t>[UNVERIFIED - confirm first]</t>
+        </is>
+      </c>
       <c r="G41" s="11" t="inlineStr"/>
       <c r="H41" s="11" t="inlineStr"/>
       <c r="I41" s="9" t="inlineStr">
         <is>
-          <t>Use the names these offices go by locally.</t>
+          <t>Marker after a contact that could not be confirmed. Keep the brackets.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="48" customHeight="1">
-      <c r="A42" s="12" t="inlineStr">
-        <is>
-          <t>E15</t>
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>E14</t>
         </is>
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>Notices</t>
+          <t>What to do</t>
         </is>
       </c>
       <c r="C42" s="9" t="inlineStr">
@@ -2084,29 +2192,29 @@
           <t>always</t>
         </is>
       </c>
-      <c r="D42" s="13" t="inlineStr">
-        <is>
-          <t>SAFETY-CRITICAL</t>
-        </is>
-      </c>
-      <c r="E42" s="12" t="inlineStr">
-        <is>
-          <t>This system CANNOT tell you whether you have a valid claim. If you believe your crop was damaged, report it through the official channels within the deadline, whatever this report says.</t>
-        </is>
-      </c>
-      <c r="F42" s="10" t="inlineStr"/>
+      <c r="D42" s="9" t="inlineStr"/>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>3. Confirm the numbers above with your bank, the Common Service Centre, or the District Agriculture Officer. They could not be verified against an official page.</t>
+        </is>
+      </c>
+      <c r="F42" s="10" t="inlineStr">
+        <is>
+          <t>3. மேலே உள்ள எண்களை உங்கள் வங்கி, பொது சேவை மையம் (Common Service Centre) அல்லது மாவட்ட வேளாண்மை அலுவலரிடம் உறுதிப்படுத்துங்கள். அதிகாரப்பூர்வ இணையப் பக்கத்தில் இவற்றை உறுதிப்படுத்த முடியவில்லை.</t>
+        </is>
+      </c>
       <c r="G42" s="11" t="inlineStr"/>
       <c r="H42" s="11" t="inlineStr"/>
       <c r="I42" s="9" t="inlineStr">
         <is>
-          <t>Mandatory notice. Must not be shortened.</t>
+          <t>Use the names these offices go by locally.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="48" customHeight="1">
       <c r="A43" s="12" t="inlineStr">
         <is>
-          <t>E16</t>
+          <t>E15</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr">
@@ -2126,10 +2234,14 @@
       </c>
       <c r="E43" s="12" t="inlineStr">
         <is>
-          <t>This is a research prototype. It is not connected to PMFBY, is not an insurer, and its output has no official standing.</t>
-        </is>
-      </c>
-      <c r="F43" s="10" t="inlineStr"/>
+          <t>This system CANNOT tell you whether you have a valid claim. If you believe your crop was damaged, report it through the official channels within the deadline, whatever this report says.</t>
+        </is>
+      </c>
+      <c r="F43" s="10" t="inlineStr">
+        <is>
+          <t>உங்களுக்கு செல்லுபடியாகும் காப்பீட்டுக் கோரிக்கை உள்ளதா என்பதை இந்த அமைப்பால் தீர்மானிக்க முடியாது. உங்கள் பயிர் சேதமடைந்ததாக நீங்கள் நம்பினால், இந்த அறிக்கை என்ன சொன்னாலும், காலக்கெடுவுக்குள் அதிகாரப்பூர்வ வழிகள் மூலம் அதைத் தெரிவியுங்கள்.</t>
+        </is>
+      </c>
       <c r="G43" s="11" t="inlineStr"/>
       <c r="H43" s="11" t="inlineStr"/>
       <c r="I43" s="9" t="inlineStr">
@@ -2138,10 +2250,49 @@
         </is>
       </c>
     </row>
+    <row r="44" ht="48" customHeight="1">
+      <c r="A44" s="12" t="inlineStr">
+        <is>
+          <t>E16</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>Notices</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="D44" s="13" t="inlineStr">
+        <is>
+          <t>SAFETY-CRITICAL</t>
+        </is>
+      </c>
+      <c r="E44" s="12" t="inlineStr">
+        <is>
+          <t>This is a research prototype. It is not connected to PMFBY, is not an insurer, and its output has no official standing.</t>
+        </is>
+      </c>
+      <c r="F44" s="10" t="inlineStr">
+        <is>
+          <t>இது ஒரு ஆராய்ச்சி முன்மாதிரி. இது PMFBY-யுடன் இணைக்கப்படவில்லை; இது காப்பீட்டு நிறுவனம் அல்ல; இதன் வெளியீட்டிற்கு அதிகாரப்பூர்வ அங்கீகாரம் இல்லை.</t>
+        </is>
+      </c>
+      <c r="G44" s="11" t="inlineStr"/>
+      <c r="H44" s="11" t="inlineStr"/>
+      <c r="I44" s="9" t="inlineStr">
+        <is>
+          <t>Mandatory notice. Must not be shortened.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I43"/>
+  <autoFilter ref="A1:I44"/>
   <dataValidations count="1">
-    <dataValidation sqref="G3:H43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="textLength" operator="lessThanOrEqual">
+    <dataValidation sqref="G3:H44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="textLength" operator="lessThanOrEqual">
       <formula1>2000</formula1>
     </dataValidation>
   </dataValidations>
@@ -2155,7 +2306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A111"/>
+  <dimension ref="A1:A115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -2322,206 +2473,207 @@
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Rank in this list: 3 of 20 (lowest first).</t>
+          <t xml:space="preserve">      In plain terms: this score does not reliably pick out</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="15" t="inlineStr"/>
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      which fields need more attention.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  WHAT TO DO NOW</t>
+          <t xml:space="preserve">      Rank in this list: 3 of 20 (lowest first).</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   1. If your crop was damaged, report it NOW. Do not wait for</t>
-        </is>
-      </c>
+      <c r="A28" s="15" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      any report, including this one.</t>
+          <t xml:space="preserve">  WHAT TO DO NOW</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      - localised calamity (hailstorm, landslide, inundation,</t>
+          <t xml:space="preserve">   1. If your crop was damaged, report it NOW. Do not wait for</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        cloudburst) and post-harvest loss</t>
+          <t xml:space="preserve">      any report, including this one.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        report within 72 hours of the event  [UNVERIFIED]</t>
+          <t xml:space="preserve">      - localised calamity (hailstorm, landslide, inundation,</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      - widespread loss across a notified area (e.g. drought,</t>
+          <t xml:space="preserve">        cloudburst) and post-harvest loss</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        flood)</t>
+          <t xml:space="preserve">        report within 72 hours of the event  [UNVERIFIED]</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        no individual intimation required  [UNVERIFIED]</t>
+          <t xml:space="preserve">      - widespread loss across a notified area (e.g. drought,</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   2. Contact one of these to report or to check status:</t>
+          <t xml:space="preserve">        flood)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      - Krishi Rakshak Portal &amp; Helpline (KRPH): 14447</t>
+          <t xml:space="preserve">        no individual intimation required  [UNVERIFIED]</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      - PMFBY WhatsApp: 7065514447  [UNVERIFIED - confirm first]</t>
+          <t xml:space="preserve">   2. Contact one of these to report or to check status:</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      - Crop Insurance mobile app: search 'Crop Insurance' by Govt. of India on the app store  [UNVERIFIED - confirm first]</t>
+          <t xml:space="preserve">      - Krishi Rakshak Portal &amp; Helpline (KRPH): 14447</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      - Claim status: pmfby.gov.in -&gt; Farmer Corner -&gt; Application Status  [UNVERIFIED - confirm first]</t>
+          <t xml:space="preserve">      - PMFBY WhatsApp: 7065514447  [UNVERIFIED - confirm first]</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   3. Confirm the numbers above with your bank, the Common</t>
+          <t xml:space="preserve">      - Crop Insurance mobile app: search 'Crop Insurance' by Govt. of India on the app store  [UNVERIFIED - confirm first]</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Service Centre, or the District Agriculture Officer.</t>
+          <t xml:space="preserve">      - Claim status: pmfby.gov.in -&gt; Farmer Corner -&gt; Application Status  [UNVERIFIED - confirm first]</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      They could not be verified against an official page.</t>
+          <t xml:space="preserve">   3. Confirm the numbers above with your bank, the Common</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="15" t="inlineStr"/>
+      <c r="A44" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Service Centre, or the District Agriculture Officer.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   This system CANNOT tell you whether you have a valid claim. If</t>
+          <t xml:space="preserve">      They could not be verified against an official page.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   you believe your crop was damaged, report it through the</t>
-        </is>
-      </c>
+      <c r="A46" s="15" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   official channels within the deadline, whatever this report</t>
+          <t xml:space="preserve">   This system CANNOT tell you whether you have a valid claim. If</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   says.</t>
+          <t xml:space="preserve">   you believe your crop was damaged, report it through the</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="15" t="inlineStr"/>
+      <c r="A49" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   official channels within the deadline, whatever this report</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="15" t="inlineStr">
         <is>
+          <t xml:space="preserve">   says.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="15" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="15" t="inlineStr">
+        <is>
           <t xml:space="preserve">   This is a research prototype. It is not connected to PMFBY, is</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="15" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   not an insurer, and its output has no official standing.</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="15" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="15">
+    <row r="54">
+      <c r="A54" s="15" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="15">
         <f>=================================================================</f>
         <v/>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="14" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="14" t="inlineStr">
         <is>
           <t>Field with NO harvest record, NOT flagged  (illustrative inputs; field 999 is not a real field)</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="15">
-        <f>=================================================================</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  FIELD REPORT   Field 999   Season oct-mar 2020</t>
         </is>
       </c>
     </row>
@@ -2534,338 +2686,365 @@
     <row r="60">
       <c r="A60" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Estimated yield: 1850 kg/acre</t>
+          <t xml:space="preserve">  FIELD REPORT   Field 999   Season oct-mar 2020</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Based on: satellite imagery (no past harvest on record)</t>
-        </is>
+      <c r="A61" s="15">
+        <f>=================================================================</f>
+        <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Compared with nearby fields: 101%</t>
+          <t xml:space="preserve">  Estimated yield: 1850 kg/acre</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="15" t="inlineStr"/>
+      <c r="A63" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Based on: satellite imagery (no past harvest on record)</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Not flagged by this system.</t>
+          <t xml:space="preserve">  Compared with nearby fields: 101%</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      THIS IS NOT EVIDENCE THAT YOUR CROP IS FINE.</t>
-        </is>
-      </c>
+      <c r="A65" s="15" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      This system misses losses. If you think your crop was</t>
+          <t xml:space="preserve">  Not flagged by this system.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      damaged, report it anyway.</t>
+          <t xml:space="preserve">      THIS IS NOT EVIDENCE THAT YOUR CROP IS FINE.</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="15" t="inlineStr"/>
+      <c r="A68" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      This system misses losses. If you think your crop was</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  HOW MUCH TO TRUST THIS</t>
+          <t xml:space="preserve">      damaged, report it anyway.</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      NO RELIABLE ESTIMATE. No past harvest on record, so</t>
-        </is>
-      </c>
+      <c r="A70" s="15" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      the figure above is a satellite guess. On test data it</t>
+          <t xml:space="preserve">  HOW MUCH TO TRUST THIS</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      was NOT shown to beat simply using the area average</t>
+          <t xml:space="preserve">      NO RELIABLE ESTIMATE. No past harvest on record, so</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      (gain 14 kg/acre, interval -30 to +4, includes zero).</t>
+          <t xml:space="preserve">      the figure above is a satellite guess. On test data it</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Do not act on the number itself.</t>
+          <t xml:space="preserve">      was NOT shown to beat simply using the area average</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      This warning means there is NO RECORD for this field.</t>
+          <t xml:space="preserve">      (gain 14 kg/acre, interval -30 to +4, includes zero).</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      It does NOT mean this estimate is worse than the ones</t>
+          <t xml:space="preserve">      Do not act on the number itself.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      without the warning: tested, the difference in error is</t>
+          <t xml:space="preserve">      This warning means there is NO RECORD for this field.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      +41 kg/acre, interval -58 to +130, which includes zero.</t>
+          <t xml:space="preserve">      It does NOT mean this estimate is worse than the ones</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      This system CANNOT tell whether this particular season was</t>
+          <t xml:space="preserve">      without the warning: tested, the difference in error is</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      bad for this field. That was tested and did not work:</t>
+          <t xml:space="preserve">      +41 kg/acre, interval -58 to +130, which includes zero.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      on fields that are sometimes below and sometimes above the</t>
+          <t xml:space="preserve">      This system CANNOT tell whether this particular season was</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      threshold, ranking AUROC is 0.626 [0.386, 0.887], which</t>
+          <t xml:space="preserve">      bad for this field. That was tested and did not work:</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      includes chance.</t>
+          <t xml:space="preserve">      on fields that are sometimes below and sometimes above the</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="15" t="inlineStr"/>
+      <c r="A84" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      threshold, ranking AUROC is 0.626 [0.386, 0.887], which</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  WHAT TO DO NOW</t>
+          <t xml:space="preserve">      includes chance.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   1. If your crop was damaged, report it NOW. Do not wait for</t>
+          <t xml:space="preserve">      In plain terms: this score does not reliably pick out</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      any report, including this one.</t>
+          <t xml:space="preserve">      which fields need more attention.</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      - localised calamity (hailstorm, landslide, inundation,</t>
-        </is>
-      </c>
+      <c r="A88" s="15" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        cloudburst) and post-harvest loss</t>
+          <t xml:space="preserve">  WHAT TO DO NOW</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        report within 72 hours of the event  [UNVERIFIED]</t>
+          <t xml:space="preserve">   1. If your crop was damaged, report it NOW. Do not wait for</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      - widespread loss across a notified area (e.g. drought,</t>
+          <t xml:space="preserve">      any report, including this one.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        flood)</t>
+          <t xml:space="preserve">      - localised calamity (hailstorm, landslide, inundation,</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">        no individual intimation required  [UNVERIFIED]</t>
+          <t xml:space="preserve">        cloudburst) and post-harvest loss</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   2. Contact one of these to report or to check status:</t>
+          <t xml:space="preserve">        report within 72 hours of the event  [UNVERIFIED]</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      - Krishi Rakshak Portal &amp; Helpline (KRPH): 14447</t>
+          <t xml:space="preserve">      - widespread loss across a notified area (e.g. drought,</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      - PMFBY WhatsApp: 7065514447  [UNVERIFIED - confirm first]</t>
+          <t xml:space="preserve">        flood)</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      - Crop Insurance mobile app: search 'Crop Insurance' by Govt. of India on the app store  [UNVERIFIED - confirm first]</t>
+          <t xml:space="preserve">        no individual intimation required  [UNVERIFIED]</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      - Claim status: pmfby.gov.in -&gt; Farmer Corner -&gt; Application Status  [UNVERIFIED - confirm first]</t>
+          <t xml:space="preserve">   2. Contact one of these to report or to check status:</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   3. Confirm the numbers above with your bank, the Common</t>
+          <t xml:space="preserve">      - Krishi Rakshak Portal &amp; Helpline (KRPH): 14447</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Service Centre, or the District Agriculture Officer.</t>
+          <t xml:space="preserve">      - PMFBY WhatsApp: 7065514447  [UNVERIFIED - confirm first]</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">      They could not be verified against an official page.</t>
+          <t xml:space="preserve">      - Crop Insurance mobile app: search 'Crop Insurance' by Govt. of India on the app store  [UNVERIFIED - confirm first]</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="15" t="inlineStr"/>
+      <c r="A102" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      - Claim status: pmfby.gov.in -&gt; Farmer Corner -&gt; Application Status  [UNVERIFIED - confirm first]</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   This system CANNOT tell you whether you have a valid claim. If</t>
+          <t xml:space="preserve">   3. Confirm the numbers above with your bank, the Common</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   you believe your crop was damaged, report it through the</t>
+          <t xml:space="preserve">      Service Centre, or the District Agriculture Officer.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   official channels within the deadline, whatever this report</t>
+          <t xml:space="preserve">      They could not be verified against an official page.</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   says.</t>
-        </is>
-      </c>
+      <c r="A106" s="15" t="inlineStr"/>
     </row>
     <row r="107">
-      <c r="A107" s="15" t="inlineStr"/>
+      <c r="A107" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   This system CANNOT tell you whether you have a valid claim. If</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   This is a research prototype. It is not connected to PMFBY, is</t>
+          <t xml:space="preserve">   you believe your crop was damaged, report it through the</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="15" t="inlineStr">
         <is>
+          <t xml:space="preserve">   official channels within the deadline, whatever this report</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   says.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="15" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   This is a research prototype. It is not connected to PMFBY, is</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="15" t="inlineStr">
+        <is>
           <t xml:space="preserve">   not an insurer, and its output has no official standing.</t>
         </is>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" s="15" t="inlineStr"/>
-    </row>
-    <row r="111">
-      <c r="A111" s="15">
+    <row r="114">
+      <c r="A114" s="15" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="15">
         <f>=================================================================</f>
         <v/>
       </c>
@@ -2881,7 +3060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A129"/>
+  <dimension ref="A1:A137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -2895,821 +3074,885 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="inlineStr"/>
+      <c r="A2" s="16">
+        <f>=================================================================</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  !!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!</t>
+          <t xml:space="preserve">  வயல் அறிக்கை   வயல் 999   பருவம் oct-mar 2020</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  THIS REPORT IS NOT TRANSLATED. 38 of 46 lines below are in</t>
-        </is>
+      <c r="A4" s="16">
+        <f>=================================================================</f>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  English, including every safety warning. The headings are</t>
+          <t xml:space="preserve">  மதிப்பிடப்பட்ட விளைச்சல்: 1240 கிலோ / ஏக்கர்</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  translated and the warnings are not, which can make the</t>
+          <t xml:space="preserve">  இதன் அடிப்படை: இந்த வயலின் முந்தைய அறுவடைகள்</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  report look prepared for you when it is not.</t>
+          <t xml:space="preserve">  அருகிலுள்ள வயல்களுடன் ஒப்பிடுகையில்: 72%</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Ask someone to read the English text with you, and do not</t>
-        </is>
-      </c>
+      <c r="A8" s="16" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  rely on the headings alone.</t>
+          <t xml:space="preserve">  &gt;&gt;&gt; கவனத்திற்காகக் குறிக்கப்பட்டது &lt;&lt;&lt;</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  !!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!</t>
+          <t xml:space="preserve">      இந்தப் பகுதியிலுள்ள ஒப்பீட்டளவில் குறைந்த விளைச்சல்</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      மதிப்பீடுகளில் இந்த வயலும் ஒன்று. இதைச் சரிபார்க்க வேண்டிய</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      காரணமாக எடுத்துக்கொள்ளுங்கள்; இழப்பு ஏற்பட்டுவிட்டது</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      என்பதற்கான முடிவாக அல்ல.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      இவ்வாறு குறிக்கப்படும் பெரும்பாலான வயல்களில், பெரும்பாலான</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      ஆண்டுகளில் விளைச்சல் சராசரிக்குக் கீழே இருக்கும். இந்தக்</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      குறிப்பு பொதுவாக நிலத்தின் வழக்கமான தன்மையைப் பற்றியது;</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      இந்தப் பருவத்தில் என்ன நடந்தது என்பதைப் பற்றியது அல்ல.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  இதை எவ்வளவு நம்பலாம்</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      மிதமான நம்பகத்தன்மை. இந்த வயலின் முந்தைய அறுவடைகளை</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      அடிப்படையாகக் கொண்டது. சோதனைத் தரவுகளில், இது</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      செயற்கைக்கோள் மாதிரியை விட விளைச்சலை மிகவும் நன்றாகக்</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      கணித்தது (பிழை 200 எதிராக 346 கிலோ/ஏக்கர்).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      இந்த குறிப்பிட்ட வயலில் இந்தப் பருவம் மோசமாக இருந்ததா</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      என்பதை இந்த அமைப்பால் கண்டறிய முடியாது. இதைச் சோதித்தபோது</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      பயனுள்ள முடிவு கிடைக்கவில்லை: சில பருவங்களில் வரம்புக்குக்</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      கீழும் சில பருவங்களில் மேலுமாக இருக்கும் வயல்களை</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      வரிசைப்படுத்திய மதிப்பெண் AUROC 0.626 [0.386, 0.887]. இந்த</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      இடைவெளியில் சீரற்ற தேர்வின் அளவும் அடங்குகிறது.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      பொதுவான விளக்கம்: இந்த மதிப்பெண், எந்த வயல்களுக்கு அதிக</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      கவனம் தேவை என்பதை நம்பகமாகத் தேர்ந்தெடுக்கவில்லை.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      இந்தப் பட்டியலில் உள்ள இடம்: 3 / 20 (குறைந்த மதிப்பீடு</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      முதலில்).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="16" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  இப்போது என்ன செய்ய வேண்டும்</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   1. உங்கள் பயிர் சேதமடைந்திருந்தால், அதை இப்போதே</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      தெரிவியுங்கள். இந்த அறிக்கை உட்பட எந்த அறிக்கைக்காகவும்</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      காத்திருக்க வேண்டாம்.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      - உள்ளூர்மயமான பேரிடர் (ஆலங்கட்டி மழை, நிலச்சரிவு, வெள்ளநீர்</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        புகுதல், திடீர் கனமழை) மற்றும் அறுவடைக்குப் பிந்தைய இழப்பு</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        நிகழ்வு நடந்த 72 மணி நேரத்திற்குள் தெரிவிக்கவும்  [UNVERIFIED]</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      - அறிவிக்கப்பட்ட பகுதி முழுவதும் பரவலான இழப்பு (எ.கா., வறட்சி,</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        வெள்ளம்)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        தனிப்பட்ட முறையில் தகவல் தெரிவிக்க வேண்டிய அவசியமில்லை  [UNVERIFIED]</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   2. இழப்பைத் தெரிவிக்க அல்லது நிலையை அறிய, கீழே உள்ள வழிகளில்</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      ஒன்றைத் தொடர்புகொள்ளுங்கள்:</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      - கிருஷி ரக்ஷக் போர்டல் &amp; உதவி எண் (KRPH): 14447</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      - PMFBY WhatsApp: 7065514447  [UNVERIFIED - confirm first]</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      - மொபைல் செயலி: செயலி அங்காடியில் இந்திய அரசின் 'Crop Insurance' என்று தேடுங்கள்.  [UNVERIFIED - confirm first]</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      - கோரிக்கை நிலை: pmfby.gov.in -&gt; Farmer Corner -&gt; Application Status  [UNVERIFIED - confirm first]</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   3. மேலே உள்ள எண்களை உங்கள் வங்கி, பொது சேவை மையம் (Common</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Service Centre) அல்லது மாவட்ட வேளாண்மை அலுவலரிடம்</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      உறுதிப்படுத்துங்கள். அதிகாரப்பூர்வ இணையப் பக்கத்தில்</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      இவற்றை உறுதிப்படுத்த முடியவில்லை.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="16" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   உங்களுக்கு செல்லுபடியாகும் காப்பீட்டுக் கோரிக்கை உள்ளதா என்பதை</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   இந்த அமைப்பால் தீர்மானிக்க முடியாது. உங்கள் பயிர் சேதமடைந்ததாக</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   நீங்கள் நம்பினால், இந்த அறிக்கை என்ன சொன்னாலும்,</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   காலக்கெடுவுக்குள் அதிகாரப்பூர்வ வழிகள் மூலம் அதைத்</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   தெரிவியுங்கள்.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="16" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   இது ஒரு ஆராய்ச்சி முன்மாதிரி. இது PMFBY-யுடன்</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   இணைக்கப்படவில்லை; இது காப்பீட்டு நிறுவனம் அல்ல; இதன்</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   வெளியீட்டிற்கு அதிகாரப்பூர்வ அங்கீகாரம் இல்லை.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="16" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="16">
         <f>=================================================================</f>
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  வயல் அறிக்கை   வயல் 999   பருவம் oct-mar 2020</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="16">
+    <row r="69">
+      <c r="A69" s="14" t="inlineStr">
+        <is>
+          <t>Field with NO harvest record, NOT flagged  (illustrative inputs; field 999 is not a real field)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="16">
         <f>=================================================================</f>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  மதிப்பிடப்பட்ட விளைச்சல்: 1240 kg/acre</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  அடிப்படை: இந்த வயலின் முந்தைய அறுவடைகள்</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  அருகிலுள்ள வயல்களுடன் ஒப்பிடுகையில்: 72%</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="16" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  &gt;&gt;&gt; கவனத்திற்கு குறிக்கப்பட்டுள்ளது &lt;&lt;&lt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      This field is among the lower estimates in its area.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      That is a reason to look, not a finding of loss.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      Most fields flagged this way yield below average MOST</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      YEARS. Being flagged is usually a statement about the</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      land, not about this season.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="16" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  இதை எவ்வளவு நம்பலாம்</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      Moderate. Built from this field's own past harvests,</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      which on test data predicted yield far better than the</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      satellite model (error 200 vs 346 kg/acre).</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      This system CANNOT tell whether this particular season was</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      bad for this field. That was tested and did not work:</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      on fields that are sometimes below and sometimes above the</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      threshold, ranking AUROC is 0.626 [0.386, 0.887], which</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      includes chance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      Rank in this list: 3 of 20 (lowest first).</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="16" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  இப்போது என்ன செய்வது</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   1. If your crop was damaged, report it NOW. Do not wait for</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      any report, including this one.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      - localised calamity (hailstorm, landslide, inundation,</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        cloudburst) and post-harvest loss</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        report within 72 hours of the event  [UNVERIFIED]</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      - widespread loss across a notified area (e.g. drought,</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        flood)</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        no individual intimation required  [UNVERIFIED]</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   2. Contact one of these to report or to check status:</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      - Krishi Rakshak Portal &amp; Helpline (KRPH): 14447</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      - PMFBY WhatsApp: 7065514447  [UNVERIFIED - confirm first]</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      - Crop Insurance mobile app: search 'Crop Insurance' by Govt. of India on the app store  [UNVERIFIED - confirm first]</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      - Claim status: pmfby.gov.in -&gt; Farmer Corner -&gt; Application Status  [UNVERIFIED - confirm first]</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   3. Confirm the numbers above with your bank, the Common</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      Service Centre, or the District Agriculture Officer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      They could not be verified against an official page.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="16" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   This system CANNOT tell you whether you have a valid claim. If</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   you believe your crop was damaged, report it through the</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   official channels within the deadline, whatever this report</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   says.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="16" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   This is a research prototype. It is not connected to PMFBY, is</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   not an insurer, and its output has no official standing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="16" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="16">
+    <row r="71">
+      <c r="A71" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  வயல் அறிக்கை   வயல் 999   பருவம் oct-mar 2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="16">
         <f>=================================================================</f>
         <v/>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="14" t="inlineStr">
-        <is>
-          <t>Field with NO harvest record, NOT flagged  (illustrative inputs; field 999 is not a real field)</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="16" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  !!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  THIS REPORT IS NOT TRANSLATED. 38 of 46 lines below are in</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  English, including every safety warning. The headings are</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  translated and the warnings are not, which can make the</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  report look prepared for you when it is not.</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Ask someone to read the English text with you, and do not</t>
-        </is>
-      </c>
-    </row>
     <row r="73">
       <c r="A73" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  rely on the headings alone.</t>
+          <t xml:space="preserve">  மதிப்பிடப்பட்ட விளைச்சல்: 1850 கிலோ / ஏக்கர்</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  !!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!</t>
+          <t xml:space="preserve">  இதன் அடிப்படை: செயற்கைக்கோள் படங்கள் (முந்தைய அறுவடைப் பதிவு இல்லை)</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="16">
-        <f>=================================================================</f>
-        <v/>
+      <c r="A75" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  அருகிலுள்ள வயல்களுடன் ஒப்பிடுகையில்: 101%</t>
+        </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  வயல் அறிக்கை   வயல் 999   பருவம் oct-mar 2020</t>
-        </is>
-      </c>
+      <c r="A76" s="16" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="16">
-        <f>=================================================================</f>
-        <v/>
+      <c r="A77" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  இந்த அமைப்பு இந்த வயலைக் குறிக்கவில்லை.</t>
+        </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  மதிப்பிடப்பட்ட விளைச்சல்: 1850 kg/acre</t>
+          <t xml:space="preserve">      உங்கள் பயிர் நன்றாக உள்ளது என்பதற்கான ஆதாரம் இது அல்ல.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  அடிப்படை: செயற்கைக்கோள் படம் (முந்தைய அறுவடை பதிவு இல்லை)</t>
+          <t xml:space="preserve">      இந்த அமைப்பு பயிர் இழப்புகளைத் தவறவிடுகிறது. உங்கள் பயிர்</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  அருகிலுள்ள வயல்களுடன் ஒப்பிடுகையில்: 101%</t>
+          <t xml:space="preserve">      சேதமடைந்ததாக நீங்கள் நினைத்தால், இருந்தாலும் அதைத்</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="16" t="inlineStr"/>
+      <c r="A81" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      தெரிவியுங்கள்.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
-      <c r="A82" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  இந்த அமைப்பால் குறிக்கப்படவில்லை.</t>
-        </is>
-      </c>
+      <c r="A82" s="16" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      THIS IS NOT EVIDENCE THAT YOUR CROP IS FINE.</t>
+          <t xml:space="preserve">  இதை எவ்வளவு நம்பலாம்</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      This system misses losses. If you think your crop was</t>
+          <t xml:space="preserve">      நம்பகமான மதிப்பீடு இல்லை. முந்தைய அறுவடைப் பதிவு இல்லை;</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      damaged, report it anyway.</t>
+          <t xml:space="preserve">      எனவே மேலே உள்ள எண் செயற்கைக்கோள் தரவின் அடிப்படையிலான ஒரு</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="16" t="inlineStr"/>
+      <c r="A86" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      கணிப்பு மட்டுமே. சோதனைத் தரவுகளில், இந்தக் கணிப்பு</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  இதை எவ்வளவு நம்பலாம்</t>
+          <t xml:space="preserve">      பகுதியின் சராசரி விளைச்சலை மட்டும் பயன்படுத்துவதை விடச்</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      NO RELIABLE ESTIMATE. No past harvest on record, so</t>
+          <t xml:space="preserve">      சிறந்தது என்று நிரூபிக்கப்படவில்லை (முன்னேற்றம் 14</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      the figure above is a satellite guess. On test data it</t>
+          <t xml:space="preserve">      கிலோ/ஏக்கர்; இடைவெளி -30 முதல் +4 வரை; இதில் பூஜ்ஜியம்</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      was NOT shown to beat simply using the area average</t>
+          <t xml:space="preserve">      அடங்குகிறது). இந்த எண்ணை மட்டும் வைத்து எந்த முடிவும்</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      (gain 14 kg/acre, interval -30 to +4, includes zero).</t>
+          <t xml:space="preserve">      எடுக்க வேண்டாம்.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Do not act on the number itself.</t>
+          <t xml:space="preserve">      இந்த எச்சரிக்கை இந்த வயலுக்கு முந்தைய அறுவடைப் பதிவு இல்லை</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      This warning means there is NO RECORD for this field.</t>
+          <t xml:space="preserve">      என்பதைக் குறிக்கிறது. எச்சரிக்கை இல்லாத வயல்களைவிட இந்த</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      It does NOT mean this estimate is worse than the ones</t>
+          <t xml:space="preserve">      மதிப்பீடு மோசமானது என்று இதன் பொருள் அல்ல: சோதனையில் பிழை</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      without the warning: tested, the difference in error is</t>
+          <t xml:space="preserve">      வித்தியாசம் +41 கிலோ/ஏக்கர்; இடைவெளி -58 முதல் +130 வரை,</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      +41 kg/acre, interval -58 to +130, which includes zero.</t>
+          <t xml:space="preserve">      இதில் பூஜ்ஜியம் அடங்குகிறது.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      This system CANNOT tell whether this particular season was</t>
+          <t xml:space="preserve">      இந்த குறிப்பிட்ட வயலில் இந்தப் பருவம் மோசமாக இருந்ததா</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      bad for this field. That was tested and did not work:</t>
+          <t xml:space="preserve">      என்பதை இந்த அமைப்பால் கண்டறிய முடியாது. இதைச் சோதித்தபோது</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      on fields that are sometimes below and sometimes above the</t>
+          <t xml:space="preserve">      பயனுள்ள முடிவு கிடைக்கவில்லை: சில பருவங்களில் வரம்புக்குக்</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      threshold, ranking AUROC is 0.626 [0.386, 0.887], which</t>
+          <t xml:space="preserve">      கீழும் சில பருவங்களில் மேலுமாக இருக்கும் வயல்களை</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      includes chance.</t>
+          <t xml:space="preserve">      வரிசைப்படுத்திய மதிப்பெண் AUROC 0.626 [0.386, 0.887]. இந்த</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="16" t="inlineStr"/>
+      <c r="A102" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      இடைவெளியில் சீரற்ற தேர்வின் அளவும் அடங்குகிறது.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  இப்போது என்ன செய்வது</t>
+          <t xml:space="preserve">      பொதுவான விளக்கம்: இந்த மதிப்பெண், எந்த வயல்களுக்கு அதிக</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   1. If your crop was damaged, report it NOW. Do not wait for</t>
+          <t xml:space="preserve">      கவனம் தேவை என்பதை நம்பகமாகத் தேர்ந்தெடுக்கவில்லை.</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      any report, including this one.</t>
-        </is>
-      </c>
+      <c r="A105" s="16" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      - localised calamity (hailstorm, landslide, inundation,</t>
+          <t xml:space="preserve">  இப்போது என்ன செய்ய வேண்டும்</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">        cloudburst) and post-harvest loss</t>
+          <t xml:space="preserve">   1. உங்கள் பயிர் சேதமடைந்திருந்தால், அதை இப்போதே</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">        report within 72 hours of the event  [UNVERIFIED]</t>
+          <t xml:space="preserve">      தெரிவியுங்கள். இந்த அறிக்கை உட்பட எந்த அறிக்கைக்காகவும்</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      - widespread loss across a notified area (e.g. drought,</t>
+          <t xml:space="preserve">      காத்திருக்க வேண்டாம்.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">        flood)</t>
+          <t xml:space="preserve">      - உள்ளூர்மயமான பேரிடர் (ஆலங்கட்டி மழை, நிலச்சரிவு, வெள்ளநீர்</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">        no individual intimation required  [UNVERIFIED]</t>
+          <t xml:space="preserve">        புகுதல், திடீர் கனமழை) மற்றும் அறுவடைக்குப் பிந்தைய இழப்பு</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   2. Contact one of these to report or to check status:</t>
+          <t xml:space="preserve">        நிகழ்வு நடந்த 72 மணி நேரத்திற்குள் தெரிவிக்கவும்  [UNVERIFIED]</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      - Krishi Rakshak Portal &amp; Helpline (KRPH): 14447</t>
+          <t xml:space="preserve">      - அறிவிக்கப்பட்ட பகுதி முழுவதும் பரவலான இழப்பு (எ.கா., வறட்சி,</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      - PMFBY WhatsApp: 7065514447  [UNVERIFIED - confirm first]</t>
+          <t xml:space="preserve">        வெள்ளம்)</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      - Crop Insurance mobile app: search 'Crop Insurance' by Govt. of India on the app store  [UNVERIFIED - confirm first]</t>
+          <t xml:space="preserve">        தனிப்பட்ட முறையில் தகவல் தெரிவிக்க வேண்டிய அவசியமில்லை  [UNVERIFIED]</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      - Claim status: pmfby.gov.in -&gt; Farmer Corner -&gt; Application Status  [UNVERIFIED - confirm first]</t>
+          <t xml:space="preserve">   2. இழப்பைத் தெரிவிக்க அல்லது நிலையை அறிய, கீழே உள்ள வழிகளில்</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   3. Confirm the numbers above with your bank, the Common</t>
+          <t xml:space="preserve">      ஒன்றைத் தொடர்புகொள்ளுங்கள்:</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Service Centre, or the District Agriculture Officer.</t>
+          <t xml:space="preserve">      - கிருஷி ரக்ஷக் போர்டல் &amp; உதவி எண் (KRPH): 14447</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">      They could not be verified against an official page.</t>
+          <t xml:space="preserve">      - PMFBY WhatsApp: 7065514447  [UNVERIFIED - confirm first]</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="16" t="inlineStr"/>
+      <c r="A120" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      - மொபைல் செயலி: செயலி அங்காடியில் இந்திய அரசின் 'Crop Insurance' என்று தேடுங்கள்.  [UNVERIFIED - confirm first]</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   This system CANNOT tell you whether you have a valid claim. If</t>
+          <t xml:space="preserve">      - கோரிக்கை நிலை: pmfby.gov.in -&gt; Farmer Corner -&gt; Application Status  [UNVERIFIED - confirm first]</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   you believe your crop was damaged, report it through the</t>
+          <t xml:space="preserve">   3. மேலே உள்ள எண்களை உங்கள் வங்கி, பொது சேவை மையம் (Common</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   official channels within the deadline, whatever this report</t>
+          <t xml:space="preserve">      Service Centre) அல்லது மாவட்ட வேளாண்மை அலுவலரிடம்</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   says.</t>
+          <t xml:space="preserve">      உறுதிப்படுத்துங்கள். அதிகாரப்பூர்வ இணையப் பக்கத்தில்</t>
         </is>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="16" t="inlineStr"/>
+      <c r="A125" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      இவற்றை உறுதிப்படுத்த முடியவில்லை.</t>
+        </is>
+      </c>
     </row>
     <row r="126">
-      <c r="A126" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   This is a research prototype. It is not connected to PMFBY, is</t>
-        </is>
-      </c>
+      <c r="A126" s="16" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   not an insurer, and its output has no official standing.</t>
+          <t xml:space="preserve">   உங்களுக்கு செல்லுபடியாகும் காப்பீட்டுக் கோரிக்கை உள்ளதா என்பதை</t>
         </is>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="16" t="inlineStr"/>
+      <c r="A128" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   இந்த அமைப்பால் தீர்மானிக்க முடியாது. உங்கள் பயிர் சேதமடைந்ததாக</t>
+        </is>
+      </c>
     </row>
     <row r="129">
-      <c r="A129" s="16">
+      <c r="A129" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   நீங்கள் நம்பினால், இந்த அறிக்கை என்ன சொன்னாலும்,</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   காலக்கெடுவுக்குள் அதிகாரப்பூர்வ வழிகள் மூலம் அதைத்</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   தெரிவியுங்கள்.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="16" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   இது ஒரு ஆராய்ச்சி முன்மாதிரி. இது PMFBY-யுடன்</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   இணைக்கப்படவில்லை; இது காப்பீட்டு நிறுவனம் அல்ல; இதன்</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   வெளியீட்டிற்கு அதிகாரப்பூர்வ அங்கீகாரம் இல்லை.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="16" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="16">
         <f>=================================================================</f>
         <v/>
       </c>

</xml_diff>